<commit_message>
feat: update tenant registry and payment history handling with detailed tenancy types and improved data structure
</commit_message>
<xml_diff>
--- a/inputs/payment-history.xlsx
+++ b/inputs/payment-history.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -596,11 +596,11 @@
       <c r="G6">
         <v>7</v>
       </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <v/>
+      <c r="H6">
+        <v>1467</v>
+      </c>
+      <c r="I6">
+        <v>583</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -631,11 +631,11 @@
       <c r="G7">
         <v>7</v>
       </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v/>
+      <c r="H7">
+        <v>1467</v>
+      </c>
+      <c r="I7">
+        <v>583</v>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -666,11 +666,11 @@
       <c r="G8">
         <v>10</v>
       </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-      <c r="I8" t="str">
-        <v/>
+      <c r="H8">
+        <v>2050</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -701,23 +701,81 @@
       <c r="G9">
         <v>9</v>
       </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
-        <v/>
+      <c r="H9">
+        <v>2050</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
       </c>
       <c r="J9" t="str">
         <v/>
       </c>
       <c r="K9" t="str">
         <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>46213</v>
+      </c>
+      <c r="B10">
+        <v>46213</v>
+      </c>
+      <c r="C10" t="str">
+        <v>מהבינלאומי ס-י</v>
+      </c>
+      <c r="D10">
+        <v>234232</v>
+      </c>
+      <c r="E10">
+        <v>1050</v>
+      </c>
+      <c r="F10" t="str">
+        <v>העברה מאת איציק אשר</v>
+      </c>
+      <c r="G10">
+        <v>8</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>46213</v>
+      </c>
+      <c r="B11">
+        <v>46213</v>
+      </c>
+      <c r="C11" t="str">
+        <v>מהבינלאומי ס-י</v>
+      </c>
+      <c r="D11">
+        <v>99086</v>
+      </c>
+      <c r="E11">
+        <v>3690</v>
+      </c>
+      <c r="F11" t="str">
+        <v>העברה מאת ניר פלג</v>
+      </c>
+      <c r="G11">
+        <v>9</v>
+      </c>
+      <c r="H11">
+        <v>2640</v>
+      </c>
+      <c r="I11">
+        <v>1050</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>